<commit_message>
Enhance PRTrack functionality by adding new variables for email and name handling in New PR.pa.yaml, improving attachment management in PR Detail.pa.yaml, and refining user role handling in Settings.pa.yaml. Update filtering logic for project lines and permissions across multiple screens to ensure accurate data representation. Additionally, include new UI elements for approver rules management, enhancing user experience and administrative capabilities.
</commit_message>
<xml_diff>
--- a/PRTrack/PRTrack-sample-data.xlsx
+++ b/PRTrack/PRTrack-sample-data.xlsx
@@ -9,15 +9,17 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="READ ME" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PRTrack - Permissions" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PRTrack - Requisitions" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PRTrack - LineItems" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PRTrack - Attachments" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PRTrack - ApproverRules" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PRTrack - NWA" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PRTrack - Requisitions" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PRTrack - LineItems" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PRTrack - Attachments" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'PRTrack - Permissions'!$A$1:$E$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'PRTrack - Requisitions'!$A$1:$R$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'PRTrack - LineItems'!$A$1:$Z$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'PRTrack - Attachments'!$A$1:$D$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'PRTrack - Requisitions'!$A$1:$R$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'PRTrack - LineItems'!$A$1:$Z$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'PRTrack - Attachments'!$A$1:$D$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -507,7 +509,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B12"/>
+  <dimension ref="A1:B22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -638,6 +640,109 @@
       <c r="B12" s="4" t="inlineStr">
         <is>
           <t>PR-001 In procurement (pending approval), PR-002 In procurement (mixed lines), PR-003 On Hold, PR-004 Draft, PR-005 Rejected.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>New lists (create in SharePoint before paste)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>PRTrack - ApproverRules</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Columns: Title (text), Project (text), Category (text), RuleType (choice: Proceed, DOA), minamount (number), maxamount (number, optional), approvername (text), approveremail (text). Paste the ApproverRules sheet. Proceed is by category. DOA is by category plus dollar band. Replace sample bands with real IOC DOA if different.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>PRTrack - NWA</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Columns: Title (NWA number, text), Project (text), nwaname (text), cbsnumber (text), cbsname (text). Paste the NWA sheet. Replace sample names with real SAP labels when you have them.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Permissions.Role</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Add choice value Project Controls. Keep Requester, Buyer, Approver, Viewer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>LineItems new columns</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Add single line text: nwaname, cbsnumber, cbsname. Add stage choice: PO creation. Keep existing nwacode, origbudget, rembudget, quoted.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Requisitions.prstatus</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Add choice value Pending PO. Keep Draft, Submitted, In procurement, Approved, Rejected, On Hold.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Attachments list</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Already exists. App now reads it for chips. After paste, attach the real file on each SharePoint item if you want files, not just names.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Paste order</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>1) Permissions  2) ApproverRules  3) NWA  4) Requisitions  5) LineItems  6) Attachments.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Studio data sources</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Add PRTrack - ApproverRules and PRTrack - NWA as SharePoint data sources, then re-export the seed .msapp so pack can see them.</t>
         </is>
       </c>
     </row>
@@ -655,7 +760,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -962,6 +1067,33 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>pc.controls@halrt.ca</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>PC Controls</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>HaLRT</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Project Controls</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:E1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -970,6 +1102,579 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
+    <col width="28" customWidth="1" min="6" max="6"/>
+    <col width="28" customWidth="1" min="7" max="7"/>
+    <col width="28" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Title</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Project</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>RuleType</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>minamount</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>maxamount</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>approvername</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>approveremail</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>HaLRT-Proceed-Engineering</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>HaLRT</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Engineering/Subconsultant</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Proceed</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Aaron Hoag</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>aaron.hoag@halrt.ca</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>HaLRT-Proceed-General</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>HaLRT</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>General Expenses</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Proceed</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>William Schreiber</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>william.schreiber@halrt.ca</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>HaLRT-Proceed-Construction</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>HaLRT</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Construction</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Proceed</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Jeff Peroff</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>jeff.peroff@halrt.ca</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>HaLRT-DOA-Eng-0-50k</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>HaLRT</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Engineering/Subconsultant</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>DOA</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" t="n">
+        <v>50000</v>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Aaron Hoag</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>aaron.hoag@halrt.ca</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>HaLRT-DOA-Eng-50k</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>HaLRT</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Engineering/Subconsultant</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>DOA</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>50000</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Tom Nierodzik</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>tom.nierodzik@halrt.ca</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>HaLRT-DOA-Gen-0-10k</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>HaLRT</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>General Expenses</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>DOA</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" t="n">
+        <v>10000</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>William Schreiber</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>william.schreiber@halrt.ca</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>HaLRT-DOA-Gen-10k</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>HaLRT</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>General Expenses</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>DOA</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>10000</v>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Tom Nierodzik</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>tom.nierodzik@halrt.ca</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>HaLRT-DOA-Con-0-100k</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>HaLRT</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Construction</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>DOA</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" t="n">
+        <v>100000</v>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Jeff Peroff</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>jeff.peroff@halrt.ca</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>HaLRT-DOA-Con-100k</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>HaLRT</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Construction</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>DOA</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>100000</v>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Tom Nierodzik</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>tom.nierodzik@halrt.ca</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="36" customWidth="1" min="1" max="1"/>
+    <col width="36" customWidth="1" min="2" max="2"/>
+    <col width="36" customWidth="1" min="3" max="3"/>
+    <col width="36" customWidth="1" min="4" max="4"/>
+    <col width="36" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Title</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Project</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>nwaname</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>cbsnumber</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>cbsname</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2200-1140</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>HaLRT</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>ADA Signage Design</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>2200</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Design and Engineering</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>1100-0500</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>HaLRT</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Site Overhead and General Expenses</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>1100</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Indirect and G&amp;A</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>3300-2210</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>HaLRT</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Temporary Works - Shoring</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>3300</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Construction</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>3300-1005</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>HaLRT</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Site Establishment - Fencing</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>3300</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Construction</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2200-0980</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>HaLRT</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Geotechnical Investigation</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>2200</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Design and Engineering</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1536,13 +2241,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z10"/>
+  <dimension ref="A1:AC10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1654,17 +2359,17 @@
           <t>nwacode</t>
         </is>
       </c>
-      <c r="Q1" s="5" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>origbudget</t>
         </is>
       </c>
-      <c r="R1" s="5" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>rembudget</t>
         </is>
       </c>
-      <c r="S1" s="5" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>budgetstatus</t>
         </is>
@@ -1702,6 +2407,21 @@
       <c r="Z1" s="5" t="inlineStr">
         <is>
           <t>doacomment</t>
+        </is>
+      </c>
+      <c r="AA1" s="5" t="inlineStr">
+        <is>
+          <t>nwaname</t>
+        </is>
+      </c>
+      <c r="AB1" s="5" t="inlineStr">
+        <is>
+          <t>cbsnumber</t>
+        </is>
+      </c>
+      <c r="AC1" s="5" t="inlineStr">
+        <is>
+          <t>cbsname</t>
         </is>
       </c>
     </row>
@@ -1755,7 +2475,7 @@
       <c r="K2" s="9" t="n">
         <v>58900</v>
       </c>
-      <c r="L2" s="7" t="inlineStr"/>
+      <c r="L2" s="7" t="n"/>
       <c r="M2" s="7" t="inlineStr">
         <is>
           <t>Subconsultant</t>
@@ -1774,23 +2494,23 @@
           <t>2200-1140</t>
         </is>
       </c>
-      <c r="Q2" s="9" t="n">
+      <c r="Q2" t="n">
         <v>60000</v>
       </c>
-      <c r="R2" s="9" t="n">
+      <c r="R2" t="n">
         <v>41200</v>
       </c>
-      <c r="S2" s="7" t="inlineStr">
+      <c r="S2" t="inlineStr">
         <is>
           <t>Within Approved Budget</t>
         </is>
       </c>
-      <c r="T2" s="7" t="inlineStr">
+      <c r="T2" s="9" t="inlineStr">
         <is>
           <t>Budget confirmed against ADA design estimate.</t>
         </is>
       </c>
-      <c r="U2" s="7" t="inlineStr">
+      <c r="U2" s="9" t="inlineStr">
         <is>
           <t>Approved</t>
         </is>
@@ -1800,7 +2520,7 @@
           <t>Tom Nierodzik</t>
         </is>
       </c>
-      <c r="W2" s="7" t="inlineStr"/>
+      <c r="W2" s="7" t="n"/>
       <c r="X2" s="7" t="inlineStr">
         <is>
           <t>Pending approval</t>
@@ -1811,7 +2531,22 @@
           <t>Tom Nierodzik</t>
         </is>
       </c>
-      <c r="Z2" s="7" t="inlineStr"/>
+      <c r="Z2" s="7" t="n"/>
+      <c r="AA2" s="7" t="inlineStr">
+        <is>
+          <t>ADA Signage Design</t>
+        </is>
+      </c>
+      <c r="AB2" s="7" t="inlineStr">
+        <is>
+          <t>2200</t>
+        </is>
+      </c>
+      <c r="AC2" s="7" t="inlineStr">
+        <is>
+          <t>Design and Engineering</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
@@ -1840,7 +2575,7 @@
       <c r="F3" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="G3" s="7" t="inlineStr"/>
+      <c r="G3" s="7" t="n"/>
       <c r="H3" s="7" t="inlineStr">
         <is>
           <t>Amarachi</t>
@@ -1869,26 +2604,26 @@
           <t>PO within AD Phase estimate</t>
         </is>
       </c>
-      <c r="N3" s="7" t="inlineStr"/>
+      <c r="N3" s="7" t="n"/>
       <c r="O3" s="7" t="n"/>
       <c r="P3" s="7" t="inlineStr">
         <is>
           <t>1100-0500</t>
         </is>
       </c>
-      <c r="Q3" s="9" t="n">
+      <c r="Q3" t="n">
         <v>5000</v>
       </c>
-      <c r="R3" s="9" t="n">
+      <c r="R3" t="n">
         <v>2600</v>
       </c>
-      <c r="S3" s="7" t="inlineStr">
+      <c r="S3" t="inlineStr">
         <is>
           <t>Within Approved Budget</t>
         </is>
       </c>
-      <c r="T3" s="7" t="inlineStr"/>
-      <c r="U3" s="7" t="inlineStr">
+      <c r="T3" s="9" t="n"/>
+      <c r="U3" s="9" t="inlineStr">
         <is>
           <t>Approved</t>
         </is>
@@ -1898,7 +2633,7 @@
           <t>Tom Nierodzik</t>
         </is>
       </c>
-      <c r="W3" s="7" t="inlineStr"/>
+      <c r="W3" s="7" t="n"/>
       <c r="X3" s="7" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -1912,6 +2647,21 @@
       <c r="Z3" s="7" t="inlineStr">
         <is>
           <t>Approved.</t>
+        </is>
+      </c>
+      <c r="AA3" s="7" t="inlineStr">
+        <is>
+          <t>Site Overhead and General Expenses</t>
+        </is>
+      </c>
+      <c r="AB3" s="7" t="inlineStr">
+        <is>
+          <t>1100</t>
+        </is>
+      </c>
+      <c r="AC3" s="7" t="inlineStr">
+        <is>
+          <t>Indirect and G&amp;A</t>
         </is>
       </c>
     </row>
@@ -1942,7 +2692,7 @@
       <c r="F4" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="G4" s="7" t="inlineStr"/>
+      <c r="G4" s="7" t="n"/>
       <c r="H4" s="7" t="inlineStr">
         <is>
           <t>Amarachi</t>
@@ -1971,26 +2721,26 @@
           <t>PO within AD Phase estimate</t>
         </is>
       </c>
-      <c r="N4" s="7" t="inlineStr"/>
+      <c r="N4" s="7" t="n"/>
       <c r="O4" s="7" t="n"/>
       <c r="P4" s="7" t="inlineStr">
         <is>
           <t>1100-0500</t>
         </is>
       </c>
-      <c r="Q4" s="9" t="n">
+      <c r="Q4" t="n">
         <v>5000</v>
       </c>
-      <c r="R4" s="9" t="n">
+      <c r="R4" t="n">
         <v>2600</v>
       </c>
-      <c r="S4" s="7" t="inlineStr">
+      <c r="S4" t="inlineStr">
         <is>
           <t>Within Approved Budget</t>
         </is>
       </c>
-      <c r="T4" s="7" t="inlineStr"/>
-      <c r="U4" s="7" t="inlineStr">
+      <c r="T4" s="9" t="n"/>
+      <c r="U4" s="9" t="inlineStr">
         <is>
           <t>Approved</t>
         </is>
@@ -2000,7 +2750,7 @@
           <t>Tom Nierodzik</t>
         </is>
       </c>
-      <c r="W4" s="7" t="inlineStr"/>
+      <c r="W4" s="7" t="n"/>
       <c r="X4" s="7" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -2014,6 +2764,21 @@
       <c r="Z4" s="7" t="inlineStr">
         <is>
           <t>Approved.</t>
+        </is>
+      </c>
+      <c r="AA4" s="7" t="inlineStr">
+        <is>
+          <t>Site Overhead and General Expenses</t>
+        </is>
+      </c>
+      <c r="AB4" s="7" t="inlineStr">
+        <is>
+          <t>1100</t>
+        </is>
+      </c>
+      <c r="AC4" s="7" t="inlineStr">
+        <is>
+          <t>Indirect and G&amp;A</t>
         </is>
       </c>
     </row>
@@ -2067,7 +2832,7 @@
       <c r="K5" s="9" t="n">
         <v>300</v>
       </c>
-      <c r="L5" s="7" t="inlineStr"/>
+      <c r="L5" s="7" t="n"/>
       <c r="M5" s="7" t="inlineStr">
         <is>
           <t>PO within AD Phase estimate</t>
@@ -2086,19 +2851,19 @@
           <t>1100-0500</t>
         </is>
       </c>
-      <c r="Q5" s="9" t="n">
+      <c r="Q5" t="n">
         <v>5000</v>
       </c>
-      <c r="R5" s="9" t="n">
+      <c r="R5" t="n">
         <v>2600</v>
       </c>
-      <c r="S5" s="7" t="inlineStr">
+      <c r="S5" t="inlineStr">
         <is>
           <t>Within Approved Budget</t>
         </is>
       </c>
-      <c r="T5" s="7" t="inlineStr"/>
-      <c r="U5" s="7" t="inlineStr">
+      <c r="T5" s="9" t="n"/>
+      <c r="U5" s="9" t="inlineStr">
         <is>
           <t>Approved</t>
         </is>
@@ -2108,7 +2873,7 @@
           <t>Tom Nierodzik</t>
         </is>
       </c>
-      <c r="W5" s="7" t="inlineStr"/>
+      <c r="W5" s="7" t="n"/>
       <c r="X5" s="7" t="inlineStr">
         <is>
           <t>Pending approval</t>
@@ -2119,7 +2884,22 @@
           <t>Tom Nierodzik</t>
         </is>
       </c>
-      <c r="Z5" s="7" t="inlineStr"/>
+      <c r="Z5" s="7" t="n"/>
+      <c r="AA5" s="7" t="inlineStr">
+        <is>
+          <t>Site Overhead and General Expenses</t>
+        </is>
+      </c>
+      <c r="AB5" s="7" t="inlineStr">
+        <is>
+          <t>1100</t>
+        </is>
+      </c>
+      <c r="AC5" s="7" t="inlineStr">
+        <is>
+          <t>Indirect and G&amp;A</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="7" t="inlineStr">
@@ -2148,7 +2928,7 @@
       <c r="F6" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="G6" s="7" t="inlineStr"/>
+      <c r="G6" s="7" t="n"/>
       <c r="H6" s="7" t="inlineStr">
         <is>
           <t>Ali</t>
@@ -2167,32 +2947,32 @@
       <c r="K6" s="9" t="n">
         <v>80</v>
       </c>
-      <c r="L6" s="7" t="inlineStr"/>
+      <c r="L6" s="7" t="n"/>
       <c r="M6" s="7" t="inlineStr">
         <is>
           <t>PO within AD Phase estimate</t>
         </is>
       </c>
-      <c r="N6" s="7" t="inlineStr"/>
+      <c r="N6" s="7" t="n"/>
       <c r="O6" s="7" t="n"/>
       <c r="P6" s="7" t="inlineStr">
         <is>
           <t>1100-0500</t>
         </is>
       </c>
-      <c r="Q6" s="9" t="n">
+      <c r="Q6" t="n">
         <v>5000</v>
       </c>
-      <c r="R6" s="9" t="n">
+      <c r="R6" t="n">
         <v>2600</v>
       </c>
-      <c r="S6" s="7" t="inlineStr">
+      <c r="S6" t="inlineStr">
         <is>
           <t>Within Approved Budget</t>
         </is>
       </c>
-      <c r="T6" s="7" t="inlineStr"/>
-      <c r="U6" s="7" t="inlineStr">
+      <c r="T6" s="9" t="n"/>
+      <c r="U6" s="9" t="inlineStr">
         <is>
           <t>Approved</t>
         </is>
@@ -2202,7 +2982,7 @@
           <t>Tom Nierodzik</t>
         </is>
       </c>
-      <c r="W6" s="7" t="inlineStr"/>
+      <c r="W6" s="7" t="n"/>
       <c r="X6" s="7" t="inlineStr">
         <is>
           <t>Sourcing</t>
@@ -2213,7 +2993,22 @@
           <t>Tom Nierodzik</t>
         </is>
       </c>
-      <c r="Z6" s="7" t="inlineStr"/>
+      <c r="Z6" s="7" t="n"/>
+      <c r="AA6" s="7" t="inlineStr">
+        <is>
+          <t>Site Overhead and General Expenses</t>
+        </is>
+      </c>
+      <c r="AB6" s="7" t="inlineStr">
+        <is>
+          <t>1100</t>
+        </is>
+      </c>
+      <c r="AC6" s="7" t="inlineStr">
+        <is>
+          <t>Indirect and G&amp;A</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="7" t="inlineStr">
@@ -2242,7 +3037,7 @@
       <c r="F7" s="7" t="n">
         <v>12</v>
       </c>
-      <c r="G7" s="7" t="inlineStr"/>
+      <c r="G7" s="7" t="n"/>
       <c r="H7" s="7" t="inlineStr">
         <is>
           <t>Ali</t>
@@ -2261,7 +3056,7 @@
       <c r="K7" s="9" t="n">
         <v>420000</v>
       </c>
-      <c r="L7" s="7" t="inlineStr"/>
+      <c r="L7" s="7" t="n"/>
       <c r="M7" s="7" t="inlineStr">
         <is>
           <t>Alternative Procurement</t>
@@ -2280,23 +3075,23 @@
           <t>3300-2210</t>
         </is>
       </c>
-      <c r="Q7" s="9" t="n">
+      <c r="Q7" t="n">
         <v>620000</v>
       </c>
-      <c r="R7" s="9" t="n">
+      <c r="R7" t="n">
         <v>0</v>
       </c>
-      <c r="S7" s="7" t="inlineStr">
+      <c r="S7" t="inlineStr">
         <is>
           <t>Requires Budget Adjustment</t>
         </is>
       </c>
-      <c r="T7" s="7" t="inlineStr">
+      <c r="T7" s="9" t="inlineStr">
         <is>
           <t>Over estimate — escalated to Design &amp; Construction Segment Integration Director.</t>
         </is>
       </c>
-      <c r="U7" s="7" t="inlineStr">
+      <c r="U7" s="9" t="inlineStr">
         <is>
           <t>Approved</t>
         </is>
@@ -2306,7 +3101,7 @@
           <t>Tom Nierodzik</t>
         </is>
       </c>
-      <c r="W7" s="7" t="inlineStr"/>
+      <c r="W7" s="7" t="n"/>
       <c r="X7" s="7" t="inlineStr">
         <is>
           <t>On hold</t>
@@ -2320,6 +3115,21 @@
       <c r="Z7" s="7" t="inlineStr">
         <is>
           <t>On hold pending budget adjustment.</t>
+        </is>
+      </c>
+      <c r="AA7" s="7" t="inlineStr">
+        <is>
+          <t>Temporary Works - Shoring</t>
+        </is>
+      </c>
+      <c r="AB7" s="7" t="inlineStr">
+        <is>
+          <t>3300</t>
+        </is>
+      </c>
+      <c r="AC7" s="7" t="inlineStr">
+        <is>
+          <t>Construction</t>
         </is>
       </c>
     </row>
@@ -2373,7 +3183,7 @@
       <c r="K8" s="9" t="n">
         <v>221500</v>
       </c>
-      <c r="L8" s="7" t="inlineStr"/>
+      <c r="L8" s="7" t="n"/>
       <c r="M8" s="7" t="inlineStr">
         <is>
           <t>Alternative Procurement</t>
@@ -2390,23 +3200,23 @@
           <t>3300-2210</t>
         </is>
       </c>
-      <c r="Q8" s="9" t="n">
+      <c r="Q8" t="n">
         <v>620000</v>
       </c>
-      <c r="R8" s="9" t="n">
+      <c r="R8" t="n">
         <v>0</v>
       </c>
-      <c r="S8" s="7" t="inlineStr">
+      <c r="S8" t="inlineStr">
         <is>
           <t>Requires Budget Adjustment</t>
         </is>
       </c>
-      <c r="T8" s="7" t="inlineStr">
+      <c r="T8" s="9" t="inlineStr">
         <is>
           <t>Over estimate — escalated to Design &amp; Construction Segment Integration Director.</t>
         </is>
       </c>
-      <c r="U8" s="7" t="inlineStr">
+      <c r="U8" s="9" t="inlineStr">
         <is>
           <t>Approved</t>
         </is>
@@ -2416,7 +3226,7 @@
           <t>Tom Nierodzik</t>
         </is>
       </c>
-      <c r="W8" s="7" t="inlineStr"/>
+      <c r="W8" s="7" t="n"/>
       <c r="X8" s="7" t="inlineStr">
         <is>
           <t>On hold</t>
@@ -2430,6 +3240,21 @@
       <c r="Z8" s="7" t="inlineStr">
         <is>
           <t>On hold pending budget adjustment.</t>
+        </is>
+      </c>
+      <c r="AA8" s="7" t="inlineStr">
+        <is>
+          <t>Temporary Works - Shoring</t>
+        </is>
+      </c>
+      <c r="AB8" s="7" t="inlineStr">
+        <is>
+          <t>3300</t>
+        </is>
+      </c>
+      <c r="AC8" s="7" t="inlineStr">
+        <is>
+          <t>Construction</t>
         </is>
       </c>
     </row>
@@ -2460,43 +3285,43 @@
       <c r="F9" s="7" t="n">
         <v>300</v>
       </c>
-      <c r="G9" s="7" t="inlineStr"/>
+      <c r="G9" s="7" t="n"/>
       <c r="H9" s="7" t="inlineStr">
         <is>
           <t>Unassigned</t>
         </is>
       </c>
-      <c r="I9" s="7" t="inlineStr"/>
-      <c r="J9" s="7" t="inlineStr"/>
+      <c r="I9" s="7" t="n"/>
+      <c r="J9" s="7" t="n"/>
       <c r="K9" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="L9" s="7" t="inlineStr"/>
+      <c r="L9" s="7" t="n"/>
       <c r="M9" s="7" t="inlineStr">
         <is>
           <t>PO within AD Phase estimate</t>
         </is>
       </c>
-      <c r="N9" s="7" t="inlineStr"/>
+      <c r="N9" s="7" t="n"/>
       <c r="O9" s="7" t="n"/>
       <c r="P9" s="7" t="inlineStr">
         <is>
           <t>3300-1005</t>
         </is>
       </c>
-      <c r="Q9" s="9" t="n">
+      <c r="Q9" t="n">
         <v>22000</v>
       </c>
-      <c r="R9" s="9" t="n">
+      <c r="R9" t="n">
         <v>22000</v>
       </c>
-      <c r="S9" s="7" t="inlineStr">
+      <c r="S9" t="inlineStr">
         <is>
           <t>Within Approved Budget</t>
         </is>
       </c>
-      <c r="T9" s="7" t="inlineStr"/>
-      <c r="U9" s="7" t="inlineStr">
+      <c r="T9" s="9" t="n"/>
+      <c r="U9" s="9" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -2506,7 +3331,7 @@
           <t>Tom Nierodzik</t>
         </is>
       </c>
-      <c r="W9" s="7" t="inlineStr"/>
+      <c r="W9" s="7" t="n"/>
       <c r="X9" s="7" t="inlineStr">
         <is>
           <t>Pending proceed</t>
@@ -2517,7 +3342,22 @@
           <t>Tom Nierodzik</t>
         </is>
       </c>
-      <c r="Z9" s="7" t="inlineStr"/>
+      <c r="Z9" s="7" t="n"/>
+      <c r="AA9" s="7" t="inlineStr">
+        <is>
+          <t>Site Establishment - Fencing</t>
+        </is>
+      </c>
+      <c r="AB9" s="7" t="inlineStr">
+        <is>
+          <t>3300</t>
+        </is>
+      </c>
+      <c r="AC9" s="7" t="inlineStr">
+        <is>
+          <t>Construction</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
@@ -2569,32 +3409,32 @@
       <c r="K10" s="9" t="n">
         <v>11800</v>
       </c>
-      <c r="L10" s="7" t="inlineStr"/>
+      <c r="L10" s="7" t="n"/>
       <c r="M10" s="7" t="inlineStr">
         <is>
           <t>Subconsultant</t>
         </is>
       </c>
-      <c r="N10" s="7" t="inlineStr"/>
+      <c r="N10" s="7" t="n"/>
       <c r="O10" s="7" t="n"/>
       <c r="P10" s="7" t="inlineStr">
         <is>
           <t>2200-0980</t>
         </is>
       </c>
-      <c r="Q10" s="9" t="n">
+      <c r="Q10" t="n">
         <v>15000</v>
       </c>
-      <c r="R10" s="9" t="n">
+      <c r="R10" t="n">
         <v>3200</v>
       </c>
-      <c r="S10" s="7" t="inlineStr">
+      <c r="S10" t="inlineStr">
         <is>
           <t>Within Approved Budget</t>
         </is>
       </c>
-      <c r="T10" s="7" t="inlineStr"/>
-      <c r="U10" s="7" t="inlineStr">
+      <c r="T10" s="9" t="n"/>
+      <c r="U10" s="9" t="inlineStr">
         <is>
           <t>Approved</t>
         </is>
@@ -2604,7 +3444,7 @@
           <t>Tom Nierodzik</t>
         </is>
       </c>
-      <c r="W10" s="7" t="inlineStr"/>
+      <c r="W10" s="7" t="n"/>
       <c r="X10" s="7" t="inlineStr">
         <is>
           <t>Rejected</t>
@@ -2618,6 +3458,21 @@
       <c r="Z10" s="7" t="inlineStr">
         <is>
           <t>Duplicate of PR-003 scope.</t>
+        </is>
+      </c>
+      <c r="AA10" s="7" t="inlineStr">
+        <is>
+          <t>Geotechnical Investigation</t>
+        </is>
+      </c>
+      <c r="AB10" s="7" t="inlineStr">
+        <is>
+          <t>2200</t>
+        </is>
+      </c>
+      <c r="AC10" s="7" t="inlineStr">
+        <is>
+          <t>Design and Engineering</t>
         </is>
       </c>
     </row>
@@ -2627,7 +3482,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>